<commit_message>
Deploy: FIX FINAL v2026.2 (Credentials + Sidebar)
</commit_message>
<xml_diff>
--- a/public/templates/digital/Botiquines.xlsx
+++ b/public/templates/digital/Botiquines.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30006"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.1.252\Control_Interno\DOCUMENTOS\V. 17\EDITABLES V. 17\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jlcan\Desktop\Seguimiento de plataforma de seguridad Antigravity\ssoma-platform\public\templates\digital\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE07A538-300B-40C4-B585-7FA74BDCA111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A190E3D-C10C-4B0C-AB3C-A87975851F8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12300" windowHeight="7440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="F-SIG-030" sheetId="2" r:id="rId1"/>
@@ -31,15 +31,37 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="48">
-  <si>
-    <t xml:space="preserve">                                                                                                                                  </t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
   <si>
     <t>INSPECCIÓN DE BOTIQUÍN</t>
   </si>
@@ -226,7 +248,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0#"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -538,50 +560,59 @@
     <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -593,12 +624,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -612,9 +637,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -648,53 +670,68 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>83606</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>87840</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>599017</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="2 Imagen">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:srcRect l="3186" t="10559" r="60020" b="52795"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="83606" y="87840"/>
-          <a:ext cx="763061" cy="350310"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -985,106 +1022,106 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T48"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="3.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" style="2" customWidth="1"/>
     <col min="3" max="3" width="11" style="2" customWidth="1"/>
-    <col min="4" max="4" width="9.5703125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="4.5703125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="9.5546875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="4.5546875" style="2" customWidth="1"/>
     <col min="6" max="6" width="6" style="2" customWidth="1"/>
-    <col min="7" max="7" width="5.7109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="3.7109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="6.7109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="5.6640625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="3.6640625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="6.6640625" style="2" customWidth="1"/>
     <col min="10" max="10" width="10" style="2" customWidth="1"/>
-    <col min="11" max="13" width="6.5703125" style="2" customWidth="1"/>
-    <col min="14" max="14" width="5.7109375" style="2" customWidth="1"/>
-    <col min="15" max="15" width="4.140625" style="2" customWidth="1"/>
-    <col min="16" max="16" width="10.140625" style="2" customWidth="1"/>
-    <col min="17" max="17" width="17.7109375" style="2" customWidth="1"/>
+    <col min="11" max="13" width="6.5546875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="5.6640625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="4.109375" style="2" customWidth="1"/>
+    <col min="16" max="16" width="10.109375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="17.6640625" style="2" customWidth="1"/>
     <col min="18" max="20" width="4" style="2" customWidth="1"/>
-    <col min="21" max="21" width="12.140625" style="2" customWidth="1"/>
-    <col min="22" max="16384" width="11.42578125" style="2"/>
+    <col min="21" max="21" width="12.109375" style="2" customWidth="1"/>
+    <col min="22" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="21" customHeight="1">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="34" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="28" t="s">
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="36" t="s">
         <v>2</v>
-      </c>
-      <c r="K1" s="36" t="s">
-        <v>3</v>
       </c>
       <c r="L1" s="36"/>
       <c r="M1" s="36"/>
     </row>
-    <row r="2" spans="1:20" ht="21" customHeight="1">
+    <row r="2" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="34"/>
       <c r="B2" s="34"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="33"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="32"/>
       <c r="J2" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="K2" s="37" t="s">
         <v>4</v>
-      </c>
-      <c r="K2" s="37" t="s">
-        <v>5</v>
       </c>
       <c r="L2" s="36"/>
       <c r="M2" s="36"/>
     </row>
-    <row r="3" spans="1:20" ht="9.75" customHeight="1"/>
-    <row r="4" spans="1:20">
+    <row r="3" spans="1:20" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="13"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+    </row>
+    <row r="5" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
-      <c r="L4" s="27"/>
-      <c r="M4" s="27"/>
-    </row>
-    <row r="5" spans="1:20" s="3" customFormat="1">
-      <c r="A5" s="26" t="s">
+      <c r="B5" s="33"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="35" t="s">
-        <v>8</v>
-      </c>
       <c r="H5" s="35"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="23"/>
+      <c r="I5" s="38"/>
+      <c r="J5" s="38"/>
+      <c r="K5" s="38"/>
+      <c r="L5" s="38"/>
+      <c r="M5" s="38"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
@@ -1093,22 +1130,22 @@
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
     </row>
-    <row r="6" spans="1:20" s="3" customFormat="1" ht="24" customHeight="1">
-      <c r="A6" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="24"/>
-      <c r="K6" s="24"/>
-      <c r="L6" s="24"/>
-      <c r="M6" s="24"/>
+    <row r="6" spans="1:20" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="39"/>
+      <c r="J6" s="39"/>
+      <c r="K6" s="39"/>
+      <c r="L6" s="39"/>
+      <c r="M6" s="39"/>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
@@ -1117,22 +1154,22 @@
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
     </row>
-    <row r="7" spans="1:20" s="3" customFormat="1" ht="30" customHeight="1">
-      <c r="A7" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
+    <row r="7" spans="1:20" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="38"/>
+      <c r="G7" s="38"/>
+      <c r="H7" s="38"/>
+      <c r="I7" s="38"/>
+      <c r="J7" s="38"/>
+      <c r="K7" s="38"/>
+      <c r="L7" s="38"/>
+      <c r="M7" s="38"/>
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
@@ -1141,22 +1178,22 @@
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
     </row>
-    <row r="8" spans="1:20" s="3" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A8" s="25" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="23"/>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
+    <row r="8" spans="1:20" s="3" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="38"/>
+      <c r="I8" s="38"/>
+      <c r="J8" s="38"/>
+      <c r="K8" s="38"/>
+      <c r="L8" s="38"/>
+      <c r="M8" s="38"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
@@ -1165,7 +1202,7 @@
       <c r="S8" s="2"/>
       <c r="T8" s="2"/>
     </row>
-    <row r="9" spans="1:20" s="3" customFormat="1" ht="10.5" customHeight="1">
+    <row r="9" spans="1:20" s="3" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -1187,25 +1224,25 @@
       <c r="S9" s="2"/>
       <c r="T9" s="2"/>
     </row>
-    <row r="10" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
+    <row r="10" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
-      <c r="B10" s="38" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
+      <c r="B10" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
       <c r="J10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="L10" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="L10" s="12" t="s">
+      <c r="M10" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="M10" s="6" t="s">
-        <v>15</v>
       </c>
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
@@ -1215,42 +1252,42 @@
       <c r="S10" s="2"/>
       <c r="T10" s="2"/>
     </row>
-    <row r="11" spans="1:20">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="7"/>
-      <c r="B11" s="38" t="s">
+      <c r="B11" s="41" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
+      <c r="L11" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="L11" s="12" t="s">
+      <c r="M11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="M11" s="6" t="s">
-        <v>18</v>
-      </c>
       <c r="O11" s="1"/>
     </row>
-    <row r="12" spans="1:20" ht="15.75" customHeight="1">
+    <row r="12" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7"/>
       <c r="B12" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="43"/>
+      <c r="I12" s="43"/>
+      <c r="L12" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="40"/>
-      <c r="L12" s="12" t="s">
+      <c r="M12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M12" s="6" t="s">
-        <v>21</v>
-      </c>
       <c r="O12" s="1"/>
     </row>
-    <row r="13" spans="1:20" ht="9" customHeight="1">
+    <row r="13" spans="1:20" ht="9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -1259,45 +1296,45 @@
       <c r="K13" s="16"/>
       <c r="O13" s="1"/>
     </row>
-    <row r="14" spans="1:20" ht="18" customHeight="1">
-      <c r="A14" s="45" t="s">
+    <row r="14" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="47"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="46"/>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="47"/>
-      <c r="J14" s="19" t="s">
-        <v>23</v>
-      </c>
       <c r="K14" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M14" s="11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" s="14">
         <v>1</v>
       </c>
-      <c r="B15" s="41" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="42"/>
+      <c r="B15" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
       <c r="J15" s="20">
         <v>2</v>
       </c>
@@ -1305,20 +1342,20 @@
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
     </row>
-    <row r="16" spans="1:20">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" s="6">
         <v>2</v>
       </c>
-      <c r="B16" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="42"/>
-      <c r="G16" s="42"/>
-      <c r="H16" s="42"/>
-      <c r="I16" s="42"/>
+      <c r="B16" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
       <c r="J16" s="20">
         <v>1</v>
       </c>
@@ -1326,20 +1363,20 @@
       <c r="L16" s="5"/>
       <c r="M16" s="5"/>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>3</v>
       </c>
-      <c r="B17" s="41" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="42"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="42"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="42"/>
-      <c r="H17" s="42"/>
-      <c r="I17" s="42"/>
+      <c r="B17" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
       <c r="J17" s="20">
         <v>1</v>
       </c>
@@ -1347,20 +1384,20 @@
       <c r="L17" s="5"/>
       <c r="M17" s="5"/>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="14">
         <v>4</v>
       </c>
-      <c r="B18" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="42"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="42"/>
+      <c r="B18" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
       <c r="J18" s="20">
         <v>1</v>
       </c>
@@ -1368,20 +1405,20 @@
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>5</v>
       </c>
-      <c r="B19" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19" s="42"/>
-      <c r="D19" s="42"/>
-      <c r="E19" s="42"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="42"/>
-      <c r="I19" s="42"/>
+      <c r="B19" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="25"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="25"/>
+      <c r="H19" s="25"/>
+      <c r="I19" s="25"/>
       <c r="J19" s="20">
         <v>5</v>
       </c>
@@ -1389,20 +1426,20 @@
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="6">
         <v>6</v>
       </c>
-      <c r="B20" s="41" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="42"/>
-      <c r="I20" s="42"/>
+      <c r="B20" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="25"/>
+      <c r="H20" s="25"/>
+      <c r="I20" s="25"/>
       <c r="J20" s="20">
         <v>8</v>
       </c>
@@ -1410,20 +1447,20 @@
       <c r="L20" s="5"/>
       <c r="M20" s="5"/>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="14">
         <v>7</v>
       </c>
-      <c r="B21" s="41" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="42"/>
-      <c r="D21" s="42"/>
-      <c r="E21" s="42"/>
-      <c r="F21" s="42"/>
-      <c r="G21" s="42"/>
-      <c r="H21" s="42"/>
-      <c r="I21" s="42"/>
+      <c r="B21" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="25"/>
+      <c r="I21" s="25"/>
       <c r="J21" s="20">
         <v>1</v>
       </c>
@@ -1431,20 +1468,20 @@
       <c r="L21" s="5"/>
       <c r="M21" s="5"/>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="6">
         <v>8</v>
       </c>
-      <c r="B22" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="C22" s="42"/>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="42"/>
+      <c r="B22" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="25"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="25"/>
+      <c r="I22" s="25"/>
       <c r="J22" s="20">
         <v>2</v>
       </c>
@@ -1452,20 +1489,20 @@
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>9</v>
       </c>
-      <c r="B23" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" s="42"/>
-      <c r="D23" s="42"/>
-      <c r="E23" s="42"/>
-      <c r="F23" s="42"/>
-      <c r="G23" s="42"/>
-      <c r="H23" s="42"/>
-      <c r="I23" s="42"/>
+      <c r="B23" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="25"/>
       <c r="J23" s="20">
         <v>2</v>
       </c>
@@ -1473,20 +1510,20 @@
       <c r="L23" s="5"/>
       <c r="M23" s="5"/>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="14">
         <v>10</v>
       </c>
-      <c r="B24" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="C24" s="42"/>
-      <c r="D24" s="42"/>
-      <c r="E24" s="42"/>
-      <c r="F24" s="42"/>
-      <c r="G24" s="42"/>
-      <c r="H24" s="42"/>
-      <c r="I24" s="42"/>
+      <c r="B24" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="25"/>
+      <c r="I24" s="25"/>
       <c r="J24" s="20">
         <v>1</v>
       </c>
@@ -1494,20 +1531,20 @@
       <c r="L24" s="5"/>
       <c r="M24" s="5"/>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>11</v>
       </c>
-      <c r="B25" s="41" t="s">
-        <v>34</v>
-      </c>
-      <c r="C25" s="42"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="42"/>
-      <c r="F25" s="42"/>
-      <c r="G25" s="42"/>
-      <c r="H25" s="42"/>
-      <c r="I25" s="42"/>
+      <c r="B25" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" s="25"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="25"/>
+      <c r="I25" s="25"/>
       <c r="J25" s="20">
         <v>1</v>
       </c>
@@ -1515,20 +1552,20 @@
       <c r="L25" s="5"/>
       <c r="M25" s="5"/>
     </row>
-    <row r="26" spans="1:13" ht="17.25" customHeight="1">
+    <row r="26" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6">
         <v>12</v>
       </c>
-      <c r="B26" s="41" t="s">
-        <v>35</v>
-      </c>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="42"/>
-      <c r="F26" s="42"/>
-      <c r="G26" s="42"/>
-      <c r="H26" s="42"/>
-      <c r="I26" s="42"/>
+      <c r="B26" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
+      <c r="I26" s="25"/>
       <c r="J26" s="20">
         <v>10</v>
       </c>
@@ -1536,20 +1573,20 @@
       <c r="L26" s="5"/>
       <c r="M26" s="5"/>
     </row>
-    <row r="27" spans="1:13" ht="21" customHeight="1">
+    <row r="27" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="14">
         <v>13</v>
       </c>
-      <c r="B27" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="C27" s="44"/>
-      <c r="D27" s="44"/>
-      <c r="E27" s="44"/>
-      <c r="F27" s="44"/>
-      <c r="G27" s="44"/>
-      <c r="H27" s="44"/>
-      <c r="I27" s="44"/>
+      <c r="B27" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="45"/>
+      <c r="D27" s="45"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="45"/>
+      <c r="G27" s="45"/>
+      <c r="H27" s="45"/>
+      <c r="I27" s="45"/>
       <c r="J27" s="20">
         <v>1</v>
       </c>
@@ -1557,20 +1594,20 @@
       <c r="L27" s="5"/>
       <c r="M27" s="5"/>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="6">
         <v>14</v>
       </c>
-      <c r="B28" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="C28" s="42"/>
-      <c r="D28" s="42"/>
-      <c r="E28" s="42"/>
-      <c r="F28" s="42"/>
-      <c r="G28" s="42"/>
-      <c r="H28" s="42"/>
-      <c r="I28" s="42"/>
+      <c r="B28" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="25"/>
       <c r="J28" s="20">
         <v>2</v>
       </c>
@@ -1578,20 +1615,20 @@
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>15</v>
       </c>
-      <c r="B29" s="41" t="s">
-        <v>38</v>
-      </c>
-      <c r="C29" s="42"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="42"/>
-      <c r="F29" s="42"/>
-      <c r="G29" s="42"/>
-      <c r="H29" s="42"/>
-      <c r="I29" s="42"/>
+      <c r="B29" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="25"/>
+      <c r="I29" s="25"/>
       <c r="J29" s="20">
         <v>2</v>
       </c>
@@ -1599,20 +1636,20 @@
       <c r="L29" s="5"/>
       <c r="M29" s="5"/>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="14">
         <v>16</v>
       </c>
-      <c r="B30" s="41" t="s">
-        <v>39</v>
-      </c>
-      <c r="C30" s="42"/>
-      <c r="D30" s="42"/>
-      <c r="E30" s="42"/>
-      <c r="F30" s="42"/>
-      <c r="G30" s="42"/>
-      <c r="H30" s="42"/>
-      <c r="I30" s="42"/>
+      <c r="B30" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="25"/>
       <c r="J30" s="20">
         <v>1</v>
       </c>
@@ -1620,20 +1657,20 @@
       <c r="L30" s="5"/>
       <c r="M30" s="5"/>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
         <v>17</v>
       </c>
-      <c r="B31" s="41" t="s">
-        <v>40</v>
-      </c>
-      <c r="C31" s="42"/>
-      <c r="D31" s="42"/>
-      <c r="E31" s="42"/>
-      <c r="F31" s="42"/>
-      <c r="G31" s="42"/>
-      <c r="H31" s="42"/>
-      <c r="I31" s="42"/>
+      <c r="B31" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="25"/>
+      <c r="I31" s="25"/>
       <c r="J31" s="20">
         <v>1</v>
       </c>
@@ -1641,20 +1678,20 @@
       <c r="L31" s="5"/>
       <c r="M31" s="5"/>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" s="6">
         <v>18</v>
       </c>
-      <c r="B32" s="41" t="s">
-        <v>41</v>
-      </c>
-      <c r="C32" s="42"/>
-      <c r="D32" s="42"/>
-      <c r="E32" s="42"/>
-      <c r="F32" s="42"/>
-      <c r="G32" s="42"/>
-      <c r="H32" s="42"/>
-      <c r="I32" s="48"/>
+      <c r="B32" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="25"/>
+      <c r="I32" s="40"/>
       <c r="J32" s="21">
         <v>1</v>
       </c>
@@ -1662,20 +1699,20 @@
       <c r="L32" s="5"/>
       <c r="M32" s="5"/>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" s="14">
         <v>19</v>
       </c>
-      <c r="B33" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="C33" s="42"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="42"/>
-      <c r="F33" s="42"/>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
-      <c r="I33" s="48"/>
+      <c r="B33" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="25"/>
+      <c r="I33" s="40"/>
       <c r="J33" s="22">
         <v>10</v>
       </c>
@@ -1683,9 +1720,9 @@
       <c r="L33" s="5"/>
       <c r="M33" s="5"/>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" s="50" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B35" s="51"/>
       <c r="C35" s="51"/>
@@ -1700,7 +1737,7 @@
       <c r="L35" s="51"/>
       <c r="M35" s="51"/>
     </row>
-    <row r="36" spans="1:13" ht="14.25" customHeight="1">
+    <row r="36" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="52"/>
       <c r="B36" s="52"/>
       <c r="C36" s="52"/>
@@ -1715,7 +1752,7 @@
       <c r="L36" s="52"/>
       <c r="M36" s="52"/>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" s="52"/>
       <c r="B37" s="52"/>
       <c r="C37" s="52"/>
@@ -1730,7 +1767,7 @@
       <c r="L37" s="52"/>
       <c r="M37" s="52"/>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" s="52"/>
       <c r="B38" s="52"/>
       <c r="C38" s="52"/>
@@ -1745,7 +1782,7 @@
       <c r="L38" s="52"/>
       <c r="M38" s="52"/>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" s="52"/>
       <c r="B39" s="52"/>
       <c r="C39" s="52"/>
@@ -1760,7 +1797,7 @@
       <c r="L39" s="52"/>
       <c r="M39" s="52"/>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" s="52"/>
       <c r="B40" s="52"/>
       <c r="C40" s="52"/>
@@ -1775,7 +1812,7 @@
       <c r="L40" s="52"/>
       <c r="M40" s="52"/>
     </row>
-    <row r="41" spans="1:13">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="52"/>
       <c r="B41" s="52"/>
       <c r="C41" s="52"/>
@@ -1790,7 +1827,7 @@
       <c r="L41" s="52"/>
       <c r="M41" s="52"/>
     </row>
-    <row r="42" spans="1:13">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" s="52"/>
       <c r="B42" s="52"/>
       <c r="C42" s="52"/>
@@ -1805,9 +1842,9 @@
       <c r="L42" s="52"/>
       <c r="M42" s="52"/>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" s="53" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B44" s="53"/>
       <c r="C44" s="53"/>
@@ -1822,9 +1859,9 @@
       <c r="L44" s="53"/>
       <c r="M44" s="53"/>
     </row>
-    <row r="45" spans="1:13" ht="27.75" customHeight="1">
+    <row r="45" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="49" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B45" s="49"/>
       <c r="C45" s="49"/>
@@ -1839,9 +1876,9 @@
       <c r="L45" s="49"/>
       <c r="M45" s="49"/>
     </row>
-    <row r="46" spans="1:13" ht="26.25" customHeight="1">
+    <row r="46" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="49" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B46" s="49"/>
       <c r="C46" s="49"/>
@@ -1856,9 +1893,9 @@
       <c r="L46" s="49"/>
       <c r="M46" s="49"/>
     </row>
-    <row r="47" spans="1:13" ht="36.75" customHeight="1">
+    <row r="47" spans="1:13" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="49" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B47" s="49"/>
       <c r="C47" s="49"/>
@@ -1873,14 +1910,12 @@
       <c r="L47" s="49"/>
       <c r="M47" s="49"/>
     </row>
-    <row r="48" spans="1:13" ht="25.5" customHeight="1"/>
+    <row r="48" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B31:I31"/>
     <mergeCell ref="B18:I18"/>
     <mergeCell ref="B32:I32"/>
+    <mergeCell ref="B15:I15"/>
     <mergeCell ref="A47:M47"/>
     <mergeCell ref="A35:M35"/>
     <mergeCell ref="A36:M36"/>
@@ -1893,6 +1928,10 @@
     <mergeCell ref="A42:M42"/>
     <mergeCell ref="A38:M38"/>
     <mergeCell ref="A39:M39"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="A7:C7"/>
     <mergeCell ref="B33:I33"/>
     <mergeCell ref="B28:I28"/>
     <mergeCell ref="B10:D10"/>
@@ -1908,7 +1947,7 @@
     <mergeCell ref="B22:I22"/>
     <mergeCell ref="B23:I23"/>
     <mergeCell ref="A14:I14"/>
-    <mergeCell ref="B15:I15"/>
+    <mergeCell ref="A8:C8"/>
     <mergeCell ref="B16:I16"/>
     <mergeCell ref="B17:I17"/>
     <mergeCell ref="C4:M4"/>
@@ -1924,8 +1963,6 @@
     <mergeCell ref="D6:M6"/>
     <mergeCell ref="D7:M7"/>
     <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A8:C8"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.43307086614173229" right="0.43307086614173229" top="0.47244094488188981" bottom="0.9055118110236221" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -1936,7 +1973,6 @@
 Construcción y Administración S.A.&amp;R&amp;"Arial,Normal"&amp;9Fecha de Aprobación: 05/03/2020
 Pág. &amp;P de &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2222,13 +2258,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{633C72A4-3A18-45B3-8B86-71F3F9C98444}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{633C72A4-3A18-45B3-8B86-71F3F9C98444}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5584758B-4594-4361-8C92-CAA2A20550D9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5584758B-4594-4361-8C92-CAA2A20550D9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2b230e36-0a53-4ac0-ac01-c22c1efbb34c"/>
+    <ds:schemaRef ds:uri="e841f38b-9f23-43dc-9de2-cda5176cd52a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69588663-727D-491C-8F64-54C70B6B0C84}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69588663-727D-491C-8F64-54C70B6B0C84}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e841f38b-9f23-43dc-9de2-cda5176cd52a"/>
+    <ds:schemaRef ds:uri="2b230e36-0a53-4ac0-ac01-c22c1efbb34c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>